<commit_message>
docs(sales): add Release -> Tasks cross-link in workbook
Tasks sheet grouped by release (contiguous); each release row links to its own
tasks (e.g. 'R6: 7 tasks ->'). Full bidirectional drill-down: Release <-> Sprint <-> Tasks.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sales/HUMAIN-Create-Studio-Sprint-Release.xlsx
+++ b/docs/sales/HUMAIN-Create-Studio-Sprint-Release.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sprints'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Releases'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Releases'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$I$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -592,15 +592,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -634,6 +635,11 @@
           <t>Sprint</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -666,6 +672,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>6 tasks →</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -698,6 +709,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>2 tasks →</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -730,6 +746,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>3 tasks →</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -762,6 +783,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>2 tasks →</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -794,6 +820,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>1 task →</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -826,6 +857,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>7 tasks →</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -858,6 +894,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -890,6 +931,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>1 task →</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -922,6 +968,11 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>5 tasks →</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -954,20 +1005,34 @@
           <t>Sprint 1 →</t>
         </is>
       </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>1 task →</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:G11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1358,31 +1423,31 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>CS-8</t>
+          <t>CS-11</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Conversational Chat &amp; UX</t>
+          <t>Build-Anything</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Natural messages + action row</t>
+          <t>build_site</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Replies as natural in-thread messages with Copy/Retry; no framed cards.</t>
+          <t>Builds a complete responsive site, rendered live in-chat with Open/Download.</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>BE/FE</t>
         </is>
       </c>
       <c r="F9" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -1396,14 +1461,14 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>CS-9</t>
+          <t>CS-10</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1413,21 +1478,21 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Focused chat view</t>
+          <t>Intent routing + recommendations</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Composer drops below the thread and landing rails hide once a conversation starts.</t>
+          <t>Agent decides what to build and proactively suggests next steps.</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
@@ -1441,34 +1506,34 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CS-10</t>
+          <t>CS-12</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Conversational Chat &amp; UX</t>
+          <t>Build-Anything</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Intent routing + recommendations</t>
+          <t>build_content</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Agent decides what to build and proactively suggests next steps.</t>
+          <t>Editable content card (title, body, tags) the user can edit, copy or download.</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BE/FE</t>
         </is>
       </c>
       <c r="F11" s="11" t="n">
@@ -1493,7 +1558,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>CS-11</t>
+          <t>CS-13</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -1503,12 +1568,12 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>build_site</t>
+          <t>Publish-to-module</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Builds a complete responsive site, rendered live in-chat with Open/Download.</t>
+          <t>Markdown→Lexical conversion; publishes a draft to a chosen CMS module for review.</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -1531,34 +1596,34 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R3</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CS-12</t>
+          <t>CS-18</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Build-Anything</t>
+          <t>Brand Studio</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>build_content</t>
+          <t>Recommend→view→verify→publish flow</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Editable content card (title, body, tags) the user can edit, copy or download.</t>
+          <t>AI recommends a full guideline; user reviews/edits, then publishes or downloads.</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>BE/FE</t>
+          <t>FE/BE</t>
         </is>
       </c>
       <c r="F13" s="11" t="n">
@@ -1576,38 +1641,38 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>CS-13</t>
+          <t>CS-19</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Build-Anything</t>
+          <t>Brand Studio</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Publish-to-module</t>
+          <t>Active Brand governance</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Markdown→Lexical conversion; publishes a draft to a chosen CMS module for review.</t>
+          <t>Published active brand (isActive) steers all agent generations.</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>BE/FE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="F14" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -1621,29 +1686,29 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R4</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CS-14</t>
+          <t>CS-20</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Build-Anything</t>
+          <t>Design System</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>build_video</t>
+          <t>Prompt-driven theme</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Production-ready script/storyboard with a one-click render control.</t>
+          <t>Describe a look; agent generates a full theme with live preview and apply.</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -1666,38 +1731,38 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>CS-15</t>
+          <t>CS-8</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Build-Anything</t>
+          <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>build_image</t>
+          <t>Natural messages + action row</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Generates a real image via Replicate/Flux, shown inline.</t>
+          <t>Replies as natural in-thread messages with Copy/Retry; no framed cards.</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>BE/FE</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="F16" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
@@ -1718,27 +1783,27 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CS-16</t>
+          <t>CS-9</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Build-Anything</t>
+          <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>build_brand</t>
+          <t>Focused chat view</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Verifiable brand guideline card to publish (active brand) or download.</t>
+          <t>Composer drops below the thread and landing rails hide once a conversation starts.</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>BE/FE</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="F17" s="11" t="n">
@@ -1763,7 +1828,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>CS-17</t>
+          <t>CS-14</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1773,12 +1838,12 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>build_theme</t>
+          <t>build_video</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Generates a theme (palette/font/radius) with live swatches and Apply.</t>
+          <t>Production-ready script/storyboard with a one-click render control.</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -1787,7 +1852,7 @@
         </is>
       </c>
       <c r="F18" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
@@ -1808,27 +1873,27 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CS-18</t>
+          <t>CS-15</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Brand Studio</t>
+          <t>Build-Anything</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Recommend→view→verify→publish flow</t>
+          <t>build_image</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>AI recommends a full guideline; user reviews/edits, then publishes or downloads.</t>
+          <t>Generates a real image via Replicate/Flux, shown inline.</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>FE/BE</t>
+          <t>BE/FE</t>
         </is>
       </c>
       <c r="F19" s="11" t="n">
@@ -1846,34 +1911,34 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R6</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>CS-19</t>
+          <t>CS-16</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Brand Studio</t>
+          <t>Build-Anything</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Active Brand governance</t>
+          <t>build_brand</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Published active brand (isActive) steers all agent generations.</t>
+          <t>Verifiable brand guideline card to publish (active brand) or download.</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BE/FE</t>
         </is>
       </c>
       <c r="F20" s="10" t="n">
@@ -1891,29 +1956,29 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R6</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CS-20</t>
+          <t>CS-17</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Design System</t>
+          <t>Build-Anything</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Prompt-driven theme</t>
+          <t>build_theme</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Describe a look; agent generates a full theme with live preview and apply.</t>
+          <t>Generates a theme (palette/font/radius) with live swatches and Apply.</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -1922,7 +1987,7 @@
         </is>
       </c>
       <c r="F21" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
@@ -1936,38 +2001,38 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R6</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>CS-21</t>
+          <t>CS-23</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Bilingual UI</t>
+          <t>Platform / Cost / Infra</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>EN/Arabic language switch</t>
+          <t>Render pipeline</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Sidebar toggle flips the whole UI to Arabic RTL and back; choice persists.</t>
+          <t>Replicate image/video render service + Studio proxy routes + graceful states.</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>FE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="F22" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
@@ -1981,7 +2046,7 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R6</t>
         </is>
       </c>
     </row>
@@ -2033,27 +2098,27 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>CS-23</t>
+          <t>CS-25</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Platform / Cost / Infra</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Render pipeline</t>
+          <t>Product Requirements Document</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Replicate image/video render service + Studio proxy routes + graceful states.</t>
+          <t>Customer PRD with architecture/integration diagrams and product snapshots.</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DOC</t>
         </is>
       </c>
       <c r="F24" s="10" t="n">
@@ -2071,38 +2136,38 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R8</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CS-24</t>
+          <t>CS-26</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Platform / Cost / Infra</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Deploy + verification cycles</t>
+          <t>UI/UX and User Journeys</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>9 live releases, each built, deployed and verified end-to-end.</t>
+          <t>UI/UX and per-feature user journeys with real screenshots.</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>INF</t>
+          <t>DOC</t>
         </is>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
@@ -2116,14 +2181,14 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>R1–R9</t>
+          <t>R8</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>CS-25</t>
+          <t>CS-27</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -2133,12 +2198,12 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Product Requirements Document</t>
+          <t>High-Level Architecture</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Customer PRD with architecture/integration diagrams and product snapshots.</t>
+          <t>Context, agent core, sequence, integration and deployment diagrams.</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -2168,7 +2233,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CS-26</t>
+          <t>CS-28</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2178,12 +2243,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>UI/UX and User Journeys</t>
+          <t>Combined Master Deck</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>UI/UX and per-feature user journeys with real screenshots.</t>
+          <t>All three documents in one deck — single cover + part dividers.</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
@@ -2192,7 +2257,7 @@
         </is>
       </c>
       <c r="F27" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
@@ -2213,7 +2278,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>CS-27</t>
+          <t>CS-29</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
@@ -2223,21 +2288,21 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>High-Level Architecture</t>
+          <t>Build pipeline + repo commit</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Context, agent core, sequence, integration and deployment diagrams.</t>
+          <t>Branded PDF pipeline + collateral committed to docs/sales (PR #1).</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>DOC/INF</t>
         </is>
       </c>
       <c r="F28" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
@@ -2258,31 +2323,31 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CS-28</t>
+          <t>CS-21</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Bilingual UI</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Combined Master Deck</t>
+          <t>EN/Arabic language switch</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>All three documents in one deck — single cover + part dividers.</t>
+          <t>Sidebar toggle flips the whole UI to Arabic RTL and back; choice persists.</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>FE</t>
         </is>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
@@ -2296,38 +2361,38 @@
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R9</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>CS-29</t>
+          <t>CS-24</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Platform / Cost / Infra</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Build pipeline + repo commit</t>
+          <t>Deploy + verification cycles</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Branded PDF pipeline + collateral committed to docs/sales (PR #1).</t>
+          <t>9 live releases, each built, deployed and verified end-to-end.</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>DOC/INF</t>
+          <t>INF</t>
         </is>
       </c>
       <c r="F30" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
@@ -2341,7 +2406,7 @@
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R1–R9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sales): use proper internal 'location' hyperlinks in workbook
Switch from external-mode '#Sheet!Cell' rels to the canonical location attribute so
Release<->Sprint<->Tasks navigation works reliably in Excel, Numbers, Sheets and LibreOffice.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sales/HUMAIN-Create-Studio-Sprint-Release.xlsx
+++ b/docs/sales/HUMAIN-Create-Studio-Sprint-Release.xlsx
@@ -579,8 +579,8 @@
   </sheetData>
   <autoFilter ref="A1:G2"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId2"/>
+    <hyperlink ref="E2" location="Tasks!A1" display="29 tasks →"/>
+    <hyperlink ref="F2" location="Releases!A1" display="9 releases →"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1014,25 +1014,25 @@
   </sheetData>
   <autoFilter ref="A1:G11"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId19"/>
+    <hyperlink ref="F2" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G2" location="Tasks!A2" display="6 tasks →"/>
+    <hyperlink ref="F3" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G3" location="Tasks!A8" display="2 tasks →"/>
+    <hyperlink ref="F4" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G4" location="Tasks!A10" display="3 tasks →"/>
+    <hyperlink ref="F5" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G5" location="Tasks!A13" display="2 tasks →"/>
+    <hyperlink ref="F6" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G6" location="Tasks!A15" display="1 task →"/>
+    <hyperlink ref="F7" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G7" location="Tasks!A16" display="7 tasks →"/>
+    <hyperlink ref="F8" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F9" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G9" location="Tasks!A23" display="1 task →"/>
+    <hyperlink ref="F10" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G10" location="Tasks!A24" display="5 tasks →"/>
+    <hyperlink ref="F11" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="G11" location="Tasks!A29" display="1 task →"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2413,64 +2413,64 @@
   </sheetData>
   <autoFilter ref="A1:I30"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId58"/>
+    <hyperlink ref="H2" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I2" location="Releases!A2" display="R1"/>
+    <hyperlink ref="H3" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I3" location="Releases!A2" display="R1"/>
+    <hyperlink ref="H4" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I4" location="Releases!A2" display="R1"/>
+    <hyperlink ref="H5" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I5" location="Releases!A2" display="R1"/>
+    <hyperlink ref="H6" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I6" location="Releases!A2" display="R1"/>
+    <hyperlink ref="H7" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I7" location="Releases!A2" display="R1"/>
+    <hyperlink ref="H8" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I8" location="Releases!A3" display="R2"/>
+    <hyperlink ref="H9" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I9" location="Releases!A3" display="R2"/>
+    <hyperlink ref="H10" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I10" location="Releases!A4" display="R3"/>
+    <hyperlink ref="H11" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I11" location="Releases!A4" display="R3"/>
+    <hyperlink ref="H12" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I12" location="Releases!A4" display="R3"/>
+    <hyperlink ref="H13" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I13" location="Releases!A5" display="R4"/>
+    <hyperlink ref="H14" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I14" location="Releases!A5" display="R4"/>
+    <hyperlink ref="H15" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I15" location="Releases!A6" display="R5"/>
+    <hyperlink ref="H16" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I16" location="Releases!A7" display="R6"/>
+    <hyperlink ref="H17" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I17" location="Releases!A7" display="R6"/>
+    <hyperlink ref="H18" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I18" location="Releases!A7" display="R6"/>
+    <hyperlink ref="H19" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I19" location="Releases!A7" display="R6"/>
+    <hyperlink ref="H20" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I20" location="Releases!A7" display="R6"/>
+    <hyperlink ref="H21" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I21" location="Releases!A7" display="R6"/>
+    <hyperlink ref="H22" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I22" location="Releases!A7" display="R6"/>
+    <hyperlink ref="H23" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I23" location="Releases!A9" display="R7"/>
+    <hyperlink ref="H24" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I24" location="Releases!A10" display="R8"/>
+    <hyperlink ref="H25" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I25" location="Releases!A10" display="R8"/>
+    <hyperlink ref="H26" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I26" location="Releases!A10" display="R8"/>
+    <hyperlink ref="H27" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I27" location="Releases!A10" display="R8"/>
+    <hyperlink ref="H28" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I28" location="Releases!A10" display="R8"/>
+    <hyperlink ref="H29" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I29" location="Releases!A11" display="R9"/>
+    <hyperlink ref="H30" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="I30" location="Releases!A1" display="R1–R9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(sales): restructure workbook into 5 sprints tied to releases + tasks
Sprints S1-S5 each own their releases and tasks (was a single Sprint 1). Tasks grouped
by sprint then release; full Sprint<->Release<->Tasks cross-links (internal location
hyperlinks). Corrected total points to 114.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sales/HUMAIN-Create-Studio-Sprint-Release.xlsx
+++ b/docs/sales/HUMAIN-Create-Studio-Sprint-Release.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sprints'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sprints'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Releases'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$I$30</definedName>
   </definedNames>
@@ -33,12 +33,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000A5C58"/>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000563C1"/>
-      <u val="single"/>
+      <color rgb="000A5C58"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,12 +55,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B7A75"/>
+        <fgColor rgb="00F5F8F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F8F8"/>
+        <fgColor rgb="000B7A75"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,9 +90,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,27 +115,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -490,16 +484,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -515,72 +508,188 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Duration</t>
+          <t>Releases</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Tasks</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Releases</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="56" customHeight="1">
+    </row>
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sprint 1 — Agentic Studio</t>
+          <t>S1 · Agentic Foundation</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Turn the CMS into a genuinely agentic, conversational, bilingual platform — build-anything from one chat, governed and on-brand — and ship customer documentation.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>1 week · 9–15 Jun 2026</t>
+          <t>Stand up the agentic core (orchestrator + governed tools + specialists) and conversational, live-streaming chat.</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1 →</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
+          <t>6 →</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
           <t>Delivered</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>29 tasks →</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>9 releases →</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>121 / 121</t>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>S2 · Intelligent Build — Web and Content</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Intelligent intent routing; build real websites and editable, publishable content; rich rendering.</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2 →</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>5 →</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S3 · Brand and Design</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Brand Studio recommend→publish loop with active-brand governance; prompt-driven design system.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>2 →</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>3 →</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>S4 · Full Build Set and Claude-like UX</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Build video, image, brand and theme from chat; natural Claude-style messages and a focused chat view.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2 →</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>7 →</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S5 · Cost, Localization and Delivery</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Cost optimization, English/Arabic UI, customer documentation, and continuous delivery.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>3 →</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>8 →</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Delivered</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:F6"/>
   <hyperlinks>
-    <hyperlink ref="E2" location="Tasks!A1" display="29 tasks →"/>
-    <hyperlink ref="F2" location="Releases!A1" display="9 releases →"/>
+    <hyperlink ref="C2" location="Releases!A2" display="1 →"/>
+    <hyperlink ref="D2" location="Tasks!A2" display="6 →"/>
+    <hyperlink ref="C3" location="Releases!A3" display="2 →"/>
+    <hyperlink ref="D3" location="Tasks!A8" display="5 →"/>
+    <hyperlink ref="C4" location="Releases!A5" display="2 →"/>
+    <hyperlink ref="D4" location="Tasks!A13" display="3 →"/>
+    <hyperlink ref="C5" location="Releases!A7" display="2 →"/>
+    <hyperlink ref="D5" location="Tasks!A16" display="7 →"/>
+    <hyperlink ref="C6" location="Releases!A9" display="3 →"/>
+    <hyperlink ref="D6" location="Tasks!A23" display="8 →"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -598,9 +707,9 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -642,370 +751,370 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>aafdcf3</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Agentic core + conversational + live streaming</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F2" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>S1 →</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>6 tasks →</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>5e3b400</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Rich Markdown rendering + website build + recommendations</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>S2 →</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>2 tasks →</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>3876aed</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Intent router + content artifact + publish-to-module</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>S2 →</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>3 tasks →</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>262e861</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Brand Studio loop + active-brand governance</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>S3 →</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>2 tasks →</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>R5</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>7792480</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Design System — prompt-driven theme</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>S3 →</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>1 task →</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>c21fb2b</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Build set (video/image/brand/theme) + Claude-like chat UX</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>7 tasks →</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>R6.1</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>249a98d</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Brand-guideline palette fix</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>f734a2a</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Cost optimization (Haiku sub-agents)</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>1 task →</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>4321000</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Customer collateral docs + build pipeline (PR #1)</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>5 tasks →</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>3a61950</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>English/Arabic UI language switcher</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1 →</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>1 task →</t>
         </is>
@@ -1014,24 +1123,24 @@
   </sheetData>
   <autoFilter ref="A1:G11"/>
   <hyperlinks>
-    <hyperlink ref="F2" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F2" location="Sprints!A2" display="S1 →"/>
     <hyperlink ref="G2" location="Tasks!A2" display="6 tasks →"/>
-    <hyperlink ref="F3" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F3" location="Sprints!A3" display="S2 →"/>
     <hyperlink ref="G3" location="Tasks!A8" display="2 tasks →"/>
-    <hyperlink ref="F4" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F4" location="Sprints!A3" display="S2 →"/>
     <hyperlink ref="G4" location="Tasks!A10" display="3 tasks →"/>
-    <hyperlink ref="F5" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F5" location="Sprints!A4" display="S3 →"/>
     <hyperlink ref="G5" location="Tasks!A13" display="2 tasks →"/>
-    <hyperlink ref="F6" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F6" location="Sprints!A4" display="S3 →"/>
     <hyperlink ref="G6" location="Tasks!A15" display="1 task →"/>
-    <hyperlink ref="F7" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F7" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="G7" location="Tasks!A16" display="7 tasks →"/>
-    <hyperlink ref="F8" location="Sprints!A2" display="Sprint 1 →"/>
-    <hyperlink ref="F9" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F8" location="Sprints!A5" display="S4 →"/>
+    <hyperlink ref="F9" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="G9" location="Tasks!A23" display="1 task →"/>
-    <hyperlink ref="F10" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F10" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="G10" location="Tasks!A24" display="5 tasks →"/>
-    <hyperlink ref="F11" location="Sprints!A2" display="Sprint 1 →"/>
+    <hyperlink ref="F11" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="G11" location="Tasks!A29" display="1 task →"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1048,13 +1157,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -1066,39 +1175,39 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Release</t>
@@ -1106,1305 +1215,1305 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>CS-1</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>S1 →</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Agentic Core</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Orchestrator agent + Claude tool-use loop</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Multi-step orchestrator that plans, calls tools and assembles the deliverable; runs on Claude Opus.</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="G2" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>CS-2</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>S1 →</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Agentic Core</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Governed tools (RAG + brand)</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>retrieve_context (pgvector RAG over HUMAIN content) and get_brand_guidelines — read-only and scoped.</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="G3" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>CS-3</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>S1 →</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Agentic Core</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Specialist agents</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Drafting, localization (EN/AR), brand-guardian, SEO, editorial, research — delegated focused sub-tasks.</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="G4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>CS-4</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>S1 →</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Agentic Core</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Per-run audit logging</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Every agent run written to the audit log (user=agent-orchestrator) for full traceability.</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="G5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>CS-5</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>S1 →</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Streaming chat endpoint (SSE)</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>/studio/chat streams tokens live for a Claude-style response.</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="G6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>CS-6</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>S1 →</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Converse-then-produce</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Asks one clarifying question when the request is ambiguous; otherwise produces.</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="G7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>CS-7</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>S2 →</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Rich Markdown rendering</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Replies render as formatted rich text (headings, lists, tables) — not raw markdown.</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="G8" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>CS-11</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>S2 →</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Build-Anything</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>build_site</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Builds a complete responsive site, rendered live in-chat with Open/Download.</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="G9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>CS-10</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>S2 →</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Intent routing + recommendations</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Agent decides what to build and proactively suggests next steps.</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="G10" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I10" s="9" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>CS-12</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>S2 →</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Build-Anything</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>build_content</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Editable content card (title, body, tags) the user can edit, copy or download.</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="G11" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>CS-13</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>S2 →</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Build-Anything</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Publish-to-module</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Markdown→Lexical conversion; publishes a draft to a chosen CMS module for review.</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="G12" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>CS-18</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>S3 →</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Brand Studio</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Recommend→view→verify→publish flow</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>AI recommends a full guideline; user reviews/edits, then publishes or downloads.</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>FE/BE</t>
         </is>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="G13" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I13" s="9" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>CS-19</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>S3 →</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Brand Studio</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Active Brand governance</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Published active brand (isActive) steers all agent generations.</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="G14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>CS-20</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>S3 →</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Prompt-driven theme</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Describe a look; agent generates a full theme with live preview and apply.</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="G15" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>R5</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>CS-8</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Natural messages + action row</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Replies as natural in-thread messages with Copy/Retry; no framed cards.</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="G16" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>CS-9</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Conversational Chat &amp; UX</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Focused chat view</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Composer drops below the thread and landing rails hide once a conversation starts.</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="G17" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>CS-14</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Build-Anything</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>build_video</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Production-ready script/storyboard with a one-click render control.</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="G18" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>CS-15</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Build-Anything</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>build_image</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Generates a real image via Replicate/Flux, shown inline.</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F19" s="11" t="n">
+      <c r="G19" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I19" s="9" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>CS-16</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Build-Anything</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>build_brand</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Verifiable brand guideline card to publish (active brand) or download.</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n">
+      <c r="G20" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>CS-17</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Build-Anything</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>build_theme</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Generates a theme (palette/font/radius) with live swatches and Apply.</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>BE/FE</t>
         </is>
       </c>
-      <c r="F21" s="11" t="n">
+      <c r="G21" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I21" s="9" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>CS-23</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>S4 →</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Platform / Cost / Infra</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Render pipeline</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Replicate image/video render service + Studio proxy routes + graceful states.</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n">
+      <c r="G22" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>CS-22</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Platform / Cost / Infra</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Cost optimization</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Sub-agents/generation on Haiku, orchestrator on Opus — ~5–10x cheaper.</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="F23" s="11" t="n">
+      <c r="G23" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I23" s="9" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>CS-25</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Product Requirements Document</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Customer PRD with architecture/integration diagrams and product snapshots.</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>DOC</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n">
+      <c r="G24" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H24" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I24" s="9" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>CS-26</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>UI/UX and User Journeys</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>UI/UX and per-feature user journeys with real screenshots.</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>DOC</t>
         </is>
       </c>
-      <c r="F25" s="11" t="n">
+      <c r="G25" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>CS-27</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>High-Level Architecture</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Context, agent core, sequence, integration and deployment diagrams.</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>DOC</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n">
+      <c r="G26" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H26" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I26" s="9" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>CS-28</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>Combined Master Deck</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>All three documents in one deck — single cover + part dividers.</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>DOC</t>
         </is>
       </c>
-      <c r="F27" s="11" t="n">
+      <c r="G27" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>CS-29</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Build pipeline + repo commit</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Branded PDF pipeline + collateral committed to docs/sales (PR #1).</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>DOC/INF</t>
         </is>
       </c>
-      <c r="F28" s="10" t="n">
+      <c r="G28" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I28" s="9" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>CS-21</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Bilingual UI</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>EN/Arabic language switch</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>Sidebar toggle flips the whole UI to Arabic RTL and back; choice persists.</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="F29" s="11" t="n">
+      <c r="G29" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I29" s="9" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>CS-24</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>S5 →</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Platform / Cost / Infra</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Deploy + verification cycles</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>9 live releases, each built, deployed and verified end-to-end.</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>9 live releases, each built, deployed and verified end-to-end (spans R1–R9).</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>INF</t>
         </is>
       </c>
-      <c r="F30" s="10" t="n">
+      <c r="G30" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="I30" s="9" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>R1–R9</t>
         </is>
@@ -2413,63 +2522,63 @@
   </sheetData>
   <autoFilter ref="A1:I30"/>
   <hyperlinks>
-    <hyperlink ref="H2" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B2" location="Sprints!A2" display="S1 →"/>
     <hyperlink ref="I2" location="Releases!A2" display="R1"/>
-    <hyperlink ref="H3" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B3" location="Sprints!A2" display="S1 →"/>
     <hyperlink ref="I3" location="Releases!A2" display="R1"/>
-    <hyperlink ref="H4" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B4" location="Sprints!A2" display="S1 →"/>
     <hyperlink ref="I4" location="Releases!A2" display="R1"/>
-    <hyperlink ref="H5" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B5" location="Sprints!A2" display="S1 →"/>
     <hyperlink ref="I5" location="Releases!A2" display="R1"/>
-    <hyperlink ref="H6" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B6" location="Sprints!A2" display="S1 →"/>
     <hyperlink ref="I6" location="Releases!A2" display="R1"/>
-    <hyperlink ref="H7" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B7" location="Sprints!A2" display="S1 →"/>
     <hyperlink ref="I7" location="Releases!A2" display="R1"/>
-    <hyperlink ref="H8" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B8" location="Sprints!A3" display="S2 →"/>
     <hyperlink ref="I8" location="Releases!A3" display="R2"/>
-    <hyperlink ref="H9" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B9" location="Sprints!A3" display="S2 →"/>
     <hyperlink ref="I9" location="Releases!A3" display="R2"/>
-    <hyperlink ref="H10" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B10" location="Sprints!A3" display="S2 →"/>
     <hyperlink ref="I10" location="Releases!A4" display="R3"/>
-    <hyperlink ref="H11" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B11" location="Sprints!A3" display="S2 →"/>
     <hyperlink ref="I11" location="Releases!A4" display="R3"/>
-    <hyperlink ref="H12" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B12" location="Sprints!A3" display="S2 →"/>
     <hyperlink ref="I12" location="Releases!A4" display="R3"/>
-    <hyperlink ref="H13" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B13" location="Sprints!A4" display="S3 →"/>
     <hyperlink ref="I13" location="Releases!A5" display="R4"/>
-    <hyperlink ref="H14" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B14" location="Sprints!A4" display="S3 →"/>
     <hyperlink ref="I14" location="Releases!A5" display="R4"/>
-    <hyperlink ref="H15" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B15" location="Sprints!A4" display="S3 →"/>
     <hyperlink ref="I15" location="Releases!A6" display="R5"/>
-    <hyperlink ref="H16" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B16" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="I16" location="Releases!A7" display="R6"/>
-    <hyperlink ref="H17" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B17" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="I17" location="Releases!A7" display="R6"/>
-    <hyperlink ref="H18" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B18" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="I18" location="Releases!A7" display="R6"/>
-    <hyperlink ref="H19" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B19" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="I19" location="Releases!A7" display="R6"/>
-    <hyperlink ref="H20" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B20" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="I20" location="Releases!A7" display="R6"/>
-    <hyperlink ref="H21" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B21" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="I21" location="Releases!A7" display="R6"/>
-    <hyperlink ref="H22" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B22" location="Sprints!A5" display="S4 →"/>
     <hyperlink ref="I22" location="Releases!A7" display="R6"/>
-    <hyperlink ref="H23" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B23" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I23" location="Releases!A9" display="R7"/>
-    <hyperlink ref="H24" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B24" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I24" location="Releases!A10" display="R8"/>
-    <hyperlink ref="H25" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B25" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I25" location="Releases!A10" display="R8"/>
-    <hyperlink ref="H26" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B26" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I26" location="Releases!A10" display="R8"/>
-    <hyperlink ref="H27" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B27" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I27" location="Releases!A10" display="R8"/>
-    <hyperlink ref="H28" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B28" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I28" location="Releases!A10" display="R8"/>
-    <hyperlink ref="H29" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B29" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I29" location="Releases!A11" display="R9"/>
-    <hyperlink ref="H30" location="Sprints!A2" display="Sprint 1"/>
+    <hyperlink ref="B30" location="Sprints!A6" display="S5 →"/>
     <hyperlink ref="I30" location="Releases!A1" display="R1–R9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>